<commit_message>
docs(tilicheros): add week-1 lead capture package and channel tracking
- Add CAPTACION_SEMANA_1.md: ready-to-use copy per channel (bio, pinned
  posts, Marketplace, groups, WhatsApp status, quick clips, click-to-
  WhatsApp ad) with explicit placeholders, READY/BLOCKED table, one-shot
  data request for the owner, and WhatsApp reply/close messages mapped
  to registro columns. Nothing published, sent or paid.
- Registro: 10 origin channels shared with the plan, free-text product,
  funnel by channel with ad spend only on "Anuncio pagado (Meta)", and
  unified SIN CODIGO / OTRO rule. Excel 16 recalculation: 0 errors,
  template empty.
- Canonical doc aligned with the same code rule; ads README links the
  package.
- Close board tasks T1029-a77f and T1029-1f8e with evidence.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/tilicheros/ads/kit-cliente/registro-tilichero.xlsx
+++ b/projects/tilicheros/ads/kit-cliente/registro-tilichero.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\AppData\Local\Temp\claude\C--Users-Usuario-Documents-Codex-2026-10-29-referenced-chatgpt-conversation-this-is-an-work-Altiora-Immersive-Web-Lab\07312f5f-5198-409f-81c9-36c04a037b42\scratchpad\final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD47A15-43C9-438F-A498-D4716F9CD312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4BF80F5-E98A-461E-BE6B-606DD56EFBBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="1560" windowWidth="15375" windowHeight="8325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,6 +82,20 @@
         </r>
       </text>
     </comment>
+    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>Dónde vio la publicación por primera vez, no por dónde escribe. Marketplace, grupos y estados llevan código OTRO.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -125,7 +139,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="212">
   <si>
     <t>Registro El Tilichero: fichas, consultas y resumen</t>
   </si>
@@ -196,16 +210,73 @@
     <t>Video del mouse o periférico gaming (o del accesorio que lo sustituya).</t>
   </si>
   <si>
+    <t>Regla común</t>
+  </si>
+  <si>
+    <t>El código dice de qué pieza viene la consulta; el canal dice dónde la vio.</t>
+  </si>
+  <si>
     <t>OTRO</t>
   </si>
   <si>
-    <t>Viene por otra publicación, historia o anuncio que no es de esta prueba.</t>
+    <t>Vino por una publicación sin código que sí se identifica: Marketplace, grupo, estado de WhatsApp, clip o anuncio con foto. Se anota con su canal.</t>
   </si>
   <si>
     <t>SIN CODIGO</t>
   </si>
   <si>
-    <t>No dijo código ni de dónde viene, o escribió uno que no está en la lista (por ejemplo, GAME sin número). Copiá en la nota lo que escribió.</t>
+    <t>No se sabe la pieza: no dijo código ni de qué publicación viene, aunque diga el canal («lo vi en Instagram») o que se lo recomendaron. También si escribió un código que no está en la lista (copialo en la nota). Se anota con su canal: Instagram, Facebook (página), TikTok, Recomendación o No dijo.</t>
+  </si>
+  <si>
+    <t>Canal de origen</t>
+  </si>
+  <si>
+    <t>Regla</t>
+  </si>
+  <si>
+    <t>El canal es dónde vio la publicación por primera vez, no por dónde escribe. Casi todo termina en WhatsApp, pero eso no cambia el canal.</t>
+  </si>
+  <si>
+    <t>Instagram / TikTok</t>
+  </si>
+  <si>
+    <t>Vio una publicación, reel, historia o clip sin pagar en esa red.</t>
+  </si>
+  <si>
+    <t>Facebook (página)</t>
+  </si>
+  <si>
+    <t>Vio una publicación o reel de la página de El Tilichero, sin pagar.</t>
+  </si>
+  <si>
+    <t>Facebook Marketplace</t>
+  </si>
+  <si>
+    <t>Vio la publicación en Marketplace, aunque escriba por Messenger y después pase a WhatsApp. Código: OTRO.</t>
+  </si>
+  <si>
+    <t>Grupo de Facebook</t>
+  </si>
+  <si>
+    <t>Vio la publicación en un grupo de compra y venta. Código: OTRO.</t>
+  </si>
+  <si>
+    <t>Estado de WhatsApp</t>
+  </si>
+  <si>
+    <t>Vio un estado de WhatsApp del negocio. Código: OTRO.</t>
+  </si>
+  <si>
+    <t>Anuncio pagado (Meta)</t>
+  </si>
+  <si>
+    <t>Llegó por un anuncio pagado de Facebook o Instagram, por ejemplo uno de clic a WhatsApp. Código: el de la pieza si el anuncio la usa; si no, OTRO.</t>
+  </si>
+  <si>
+    <t>Recomendación / Otro / No dijo</t>
+  </si>
+  <si>
+    <t>Recomendación: se lo recomendó alguien (código SIN CODIGO). Otro: cualquier otro origen. No dijo: no sabe o no contesta (código SIN CODIGO; no insistir).</t>
   </si>
   <si>
     <t>Alcance (Insights)</t>
@@ -559,6 +630,30 @@
     <t>Leído el (fecha)</t>
   </si>
   <si>
+    <t>Embudo por canal de origen</t>
+  </si>
+  <si>
+    <t>Mismo filtro Desde/Hasta y misma regla de repetidas que el embudo por código. Cuenta las consultas con código de pieza (OTRO y SIN CODIGO incluidos).</t>
+  </si>
+  <si>
+    <t>La pauta de este cuadro y la del embudo por código NO se suman: es el mismo gasto visto de dos formas. Anotala en un solo lugar:</t>
+  </si>
+  <si>
+    <t>si el anuncio usa una pieza con código (GAME1, GAME2, RETRO1, RGB1), en el embudo por código; si no tiene código (por ejemplo, un anuncio con foto), aquí en «Anuncio pagado (Meta)».</t>
+  </si>
+  <si>
+    <t>Recomendación</t>
+  </si>
+  <si>
+    <t>Otro</t>
+  </si>
+  <si>
+    <t>No dijo</t>
+  </si>
+  <si>
+    <t>Consultas del periodo con código pero sin canal anotado (no entran en este cuadro)</t>
+  </si>
+  <si>
     <t>Condiciones de la prueba (contestar al revisar)</t>
   </si>
   <si>
@@ -607,9 +702,6 @@
     <t>Fuera de GAM</t>
   </si>
   <si>
-    <t>No dijo</t>
-  </si>
-  <si>
     <t>Sin dato</t>
   </si>
   <si>
@@ -677,6 +769,9 @@
   </si>
   <si>
     <t>Monto anotado sin Cobrado = Sí</t>
+  </si>
+  <si>
+    <t>Filas con código pero sin canal de origen</t>
   </si>
   <si>
     <t>Consultas marcadas como repetidas (no se cuentan en ningún total)</t>
@@ -816,7 +911,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -919,6 +1014,12 @@
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -933,9 +1034,6 @@
     <xf numFmtId="168" fontId="4" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -946,18 +1044,28 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1310,7 +1418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:C48"/>
+  <dimension ref="B1:C59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1431,20 +1539,20 @@
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B22" s="3" t="s">
+    <row r="21" spans="2:3" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="B21" s="8" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="23" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="B23" s="8" t="s">
+      <c r="C21" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="5" t="s">
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B23" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="24" spans="2:3" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B24" s="8" t="s">
         <v>30</v>
       </c>
@@ -1452,7 +1560,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B25" s="8" t="s">
         <v>32</v>
       </c>
@@ -1460,98 +1568,98 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B27" s="3" t="s">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B26" s="8" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="28" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="C26" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B27" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28" s="8" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B30" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B29" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="30" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B30" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B31" s="8" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B32" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B33" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B33" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B34" s="8" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" ht="38.25" x14ac:dyDescent="0.25">
       <c r="B35" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B36" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B39" s="8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B40" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="41" spans="2:3" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="B41" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C41" s="5" t="s">
+    </row>
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B41" s="3" t="s">
         <v>56</v>
       </c>
     </row>
@@ -1563,7 +1671,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43" s="8" t="s">
         <v>59</v>
       </c>
@@ -1571,33 +1679,110 @@
         <v>60</v>
       </c>
     </row>
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B44" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B45" s="3" t="s">
-        <v>61</v>
+      <c r="B45" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46" s="8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="47" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
       <c r="B47" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B48" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>67</v>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="49" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B49" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="50" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B50" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="51" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B51" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="2:3" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="B52" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B53" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="54" spans="2:3" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="B54" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C54" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B56" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B57" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="C57" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="58" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B58" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="59" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B59" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1665,319 +1850,319 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:68" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="53" t="s">
-        <v>68</v>
-      </c>
-      <c r="B1" s="53" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1" s="53" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="53" t="s">
-        <v>71</v>
-      </c>
-      <c r="E1" s="53" t="s">
-        <v>72</v>
-      </c>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="51" t="s">
-        <v>73</v>
-      </c>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="53" t="s">
-        <v>74</v>
-      </c>
-      <c r="N1" s="52"/>
-      <c r="O1" s="52"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="51" t="s">
-        <v>75</v>
-      </c>
-      <c r="R1" s="52"/>
-      <c r="S1" s="52"/>
-      <c r="T1" s="52"/>
-      <c r="U1" s="54" t="s">
-        <v>76</v>
-      </c>
-      <c r="V1" s="52"/>
-      <c r="W1" s="52"/>
-      <c r="X1" s="52"/>
-      <c r="Y1" s="51" t="s">
-        <v>77</v>
-      </c>
-      <c r="Z1" s="52"/>
-      <c r="AA1" s="52"/>
-      <c r="AB1" s="52"/>
-      <c r="AC1" s="53" t="s">
-        <v>78</v>
-      </c>
-      <c r="AD1" s="52"/>
-      <c r="AE1" s="52"/>
-      <c r="AF1" s="52"/>
-      <c r="AG1" s="51" t="s">
-        <v>79</v>
-      </c>
-      <c r="AH1" s="52"/>
-      <c r="AI1" s="52"/>
-      <c r="AJ1" s="52"/>
-      <c r="AK1" s="53" t="s">
-        <v>80</v>
-      </c>
-      <c r="AL1" s="52"/>
-      <c r="AM1" s="52"/>
-      <c r="AN1" s="52"/>
-      <c r="AO1" s="51" t="s">
-        <v>81</v>
-      </c>
-      <c r="AP1" s="52"/>
-      <c r="AQ1" s="52"/>
-      <c r="AR1" s="52"/>
-      <c r="AS1" s="53" t="s">
-        <v>82</v>
-      </c>
-      <c r="AT1" s="52"/>
-      <c r="AU1" s="52"/>
-      <c r="AV1" s="52"/>
-      <c r="AW1" s="51" t="s">
-        <v>83</v>
-      </c>
-      <c r="AX1" s="52"/>
-      <c r="AY1" s="52"/>
-      <c r="AZ1" s="52"/>
-      <c r="BA1" s="53" t="s">
-        <v>84</v>
-      </c>
-      <c r="BB1" s="52"/>
-      <c r="BC1" s="52"/>
-      <c r="BD1" s="52"/>
-      <c r="BE1" s="51" t="s">
-        <v>85</v>
-      </c>
-      <c r="BF1" s="52"/>
-      <c r="BG1" s="52"/>
-      <c r="BH1" s="52"/>
-      <c r="BI1" s="53" t="s">
-        <v>86</v>
-      </c>
-      <c r="BJ1" s="52"/>
-      <c r="BK1" s="52"/>
-      <c r="BL1" s="52"/>
-      <c r="BM1" s="51" t="s">
+      <c r="A1" s="54" t="s">
         <v>87</v>
       </c>
-      <c r="BN1" s="52"/>
-      <c r="BO1" s="52"/>
-      <c r="BP1" s="52"/>
+      <c r="B1" s="54" t="s">
+        <v>88</v>
+      </c>
+      <c r="C1" s="54" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" s="54" t="s">
+        <v>90</v>
+      </c>
+      <c r="E1" s="54" t="s">
+        <v>91</v>
+      </c>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="52" t="s">
+        <v>92</v>
+      </c>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="54" t="s">
+        <v>93</v>
+      </c>
+      <c r="N1" s="53"/>
+      <c r="O1" s="53"/>
+      <c r="P1" s="53"/>
+      <c r="Q1" s="52" t="s">
+        <v>94</v>
+      </c>
+      <c r="R1" s="53"/>
+      <c r="S1" s="53"/>
+      <c r="T1" s="53"/>
+      <c r="U1" s="55" t="s">
+        <v>95</v>
+      </c>
+      <c r="V1" s="53"/>
+      <c r="W1" s="53"/>
+      <c r="X1" s="53"/>
+      <c r="Y1" s="52" t="s">
+        <v>96</v>
+      </c>
+      <c r="Z1" s="53"/>
+      <c r="AA1" s="53"/>
+      <c r="AB1" s="53"/>
+      <c r="AC1" s="54" t="s">
+        <v>97</v>
+      </c>
+      <c r="AD1" s="53"/>
+      <c r="AE1" s="53"/>
+      <c r="AF1" s="53"/>
+      <c r="AG1" s="52" t="s">
+        <v>98</v>
+      </c>
+      <c r="AH1" s="53"/>
+      <c r="AI1" s="53"/>
+      <c r="AJ1" s="53"/>
+      <c r="AK1" s="54" t="s">
+        <v>99</v>
+      </c>
+      <c r="AL1" s="53"/>
+      <c r="AM1" s="53"/>
+      <c r="AN1" s="53"/>
+      <c r="AO1" s="52" t="s">
+        <v>100</v>
+      </c>
+      <c r="AP1" s="53"/>
+      <c r="AQ1" s="53"/>
+      <c r="AR1" s="53"/>
+      <c r="AS1" s="54" t="s">
+        <v>101</v>
+      </c>
+      <c r="AT1" s="53"/>
+      <c r="AU1" s="53"/>
+      <c r="AV1" s="53"/>
+      <c r="AW1" s="52" t="s">
+        <v>102</v>
+      </c>
+      <c r="AX1" s="53"/>
+      <c r="AY1" s="53"/>
+      <c r="AZ1" s="53"/>
+      <c r="BA1" s="54" t="s">
+        <v>103</v>
+      </c>
+      <c r="BB1" s="53"/>
+      <c r="BC1" s="53"/>
+      <c r="BD1" s="53"/>
+      <c r="BE1" s="52" t="s">
+        <v>104</v>
+      </c>
+      <c r="BF1" s="53"/>
+      <c r="BG1" s="53"/>
+      <c r="BH1" s="53"/>
+      <c r="BI1" s="54" t="s">
+        <v>105</v>
+      </c>
+      <c r="BJ1" s="53"/>
+      <c r="BK1" s="53"/>
+      <c r="BL1" s="53"/>
+      <c r="BM1" s="52" t="s">
+        <v>106</v>
+      </c>
+      <c r="BN1" s="53"/>
+      <c r="BO1" s="53"/>
+      <c r="BP1" s="53"/>
     </row>
     <row r="2" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="52"/>
-      <c r="B2" s="52"/>
-      <c r="C2" s="52"/>
-      <c r="D2" s="52"/>
+      <c r="A2" s="53"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
       <c r="E2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="J2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="N2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="O2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="P2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="U2" s="11" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="V2" s="11" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="W2" s="11" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="X2" s="11" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="Y2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="Z2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AA2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AB2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AC2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AD2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AE2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AF2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AG2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AH2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AI2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AJ2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AK2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AL2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AM2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AN2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AO2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AP2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AQ2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AR2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AS2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AT2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AU2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AV2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="AW2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="AX2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="AY2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="AZ2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="BA2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="BB2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="BC2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="BD2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="BE2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="BF2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="BG2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="BH2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="BI2" s="9" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="BJ2" s="9" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="BK2" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="BL2" s="9" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
       <c r="BM2" s="10" t="s">
-        <v>88</v>
+        <v>107</v>
       </c>
       <c r="BN2" s="10" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="BO2" s="10" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="BP2" s="10" t="s">
-        <v>91</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" spans="1:68" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>92</v>
+        <v>111</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="C3" s="12" t="str">
         <f>IF(D3=16,"COMPLETA","INCOMPLETA: faltan "&amp;(16-D3)&amp;" campos")</f>
@@ -2054,10 +2239,10 @@
     </row>
     <row r="4" spans="1:68" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>95</v>
+        <v>114</v>
       </c>
       <c r="C4" s="12" t="str">
         <f>IF(D4=16,"COMPLETA","INCOMPLETA: faltan "&amp;(16-D4)&amp;" campos")</f>
@@ -2134,10 +2319,10 @@
     </row>
     <row r="5" spans="1:68" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>96</v>
+        <v>115</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
       <c r="C5" s="12" t="str">
         <f>IF(D5=16,"COMPLETA","INCOMPLETA: faltan "&amp;(16-D5)&amp;" campos")</f>
@@ -2214,7 +2399,7 @@
     </row>
     <row r="7" spans="1:68" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>
@@ -2241,15 +2426,15 @@
     <mergeCell ref="BE1:BH1"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C5">
-    <cfRule type="expression" dxfId="6" priority="3">
+    <cfRule type="expression" dxfId="7" priority="3">
       <formula>$D3=16</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H5 L3:L5 P3:P5 T3:T5 X3:X5 AB3:AB5 AF3:AF5 AJ3:AJ5 AN3:AN5 AR3:AR5 AV3:AV5 AZ3:AZ5 BD3:BD5 BH3:BH5 BL3:BL5 BP3:BP5">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>H3="Sí"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>H3="No"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2283,7 +2468,7 @@
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
@@ -2299,49 +2484,49 @@
   <sheetData>
     <row r="1" spans="1:15" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>102</v>
+        <v>121</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>103</v>
+        <v>122</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>106</v>
+        <v>125</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>107</v>
+        <v>126</v>
       </c>
       <c r="N1" s="9" t="s">
-        <v>108</v>
+        <v>127</v>
       </c>
       <c r="O1" s="9" t="s">
-        <v>109</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -8347,10 +8532,10 @@
   </sheetData>
   <autoFilter ref="A1:O301" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <conditionalFormatting sqref="B2:O301">
-    <cfRule type="expression" dxfId="3" priority="1" stopIfTrue="1">
-      <formula>OR(AND($B2&lt;&gt;"",$D2=""),AND($D2&lt;&gt;"",$B2=""),AND($H2="Sí",$F2&lt;&gt;"GAM",$F2&lt;&gt;"Fuera de GAM"),AND($J2="Sí",$H2&lt;&gt;"Sí"),AND($K2="Sí",$J2&lt;&gt;"Sí"),AND($K2="Sí",$L2=""),AND($L2&lt;&gt;"",$K2&lt;&gt;"Sí"))</formula>
+    <cfRule type="expression" dxfId="4" priority="1" stopIfTrue="1">
+      <formula>OR(AND($B2&lt;&gt;"",$D2=""),AND($D2&lt;&gt;"",$B2=""),AND($H2="Sí",$F2&lt;&gt;"GAM",$F2&lt;&gt;"Fuera de GAM"),AND($J2="Sí",$H2&lt;&gt;"Sí"),AND($K2="Sí",$J2&lt;&gt;"Sí"),AND($K2="Sí",$L2=""),AND($L2&lt;&gt;"",$K2&lt;&gt;"Sí"),AND($D2&lt;&gt;"",$C2=""))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$G2="Sí"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8359,13 +8544,13 @@
       <formula1>DATE(2026,1,1)</formula1>
       <formula2>DATE(2030,12,31)</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí un canal de la lista." promptTitle="Canal de origen" prompt="Dónde vio la publicación. Si no lo dijo, No dijo. No insistir." sqref="C2:C301" xr:uid="{00000000-0002-0000-0200-000001000000}">
-      <formula1>"Instagram,Facebook,TikTok,Recomendación,Otro,No dijo"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí un canal de la lista." promptTitle="Canal de origen" prompt="Dónde vio la publicación por primera vez (no por dónde escribe). Marketplace aunque escriba por Messenger. Si no lo dijo: No dijo." sqref="C2:C301" xr:uid="{00000000-0002-0000-0200-000001000000}">
+      <formula1>"Instagram,Facebook (página),Facebook Marketplace,Grupo de Facebook,TikTok,Estado de WhatsApp,Anuncio pagado (Meta),Recomendación,Otro,No dijo"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí un código de la lista: GAME1, GAME2, RETRO1, RGB1, OTRO o SIN CODIGO." promptTitle="Código de pieza" prompt="El código que escribió la persona. Si no dijo código: SIN CODIGO. Si vino por otra publicación: OTRO." sqref="D2:D301" xr:uid="{00000000-0002-0000-0200-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí un código de la lista: GAME1, GAME2, RETRO1, RGB1, OTRO o SIN CODIGO." promptTitle="Código de pieza" prompt="La pieza de la que viene. Sin código ni publicación identificada (aunque diga el canal o una recomendación): SIN CODIGO. Marketplace, grupo, estado, clip o anuncio con foto: OTRO." sqref="D2:D301" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"GAME1,GAME2,RETRO1,RGB1,OTRO,SIN CODIGO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí un producto de la lista." promptTitle="Producto consultado" prompt="Lo que preguntó, aunque no coincida con el video que vio." sqref="E2:E301" xr:uid="{00000000-0002-0000-0200-000003000000}">
+    <dataValidation type="list" errorStyle="warning" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Producto fuera de la lista" error="Ese producto no está en la lista. Si es otro producto que vendés, aceptá para dejarlo escrito (nombre corto, sin datos personales)." promptTitle="Producto consultado" prompt="Elegí de la lista o escribí el producto que preguntó (nombre corto o modelo). Puede no coincidir con el video que vio." sqref="E2:E301" xr:uid="{00000000-0002-0000-0200-000003000000}">
       <formula1>"Audífonos gaming,Consola retro,Mouse o periférico,Otro producto,No dijo"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí GAM, Fuera de GAM o No dijo." promptTitle="Zona" prompt="Solo GAM, Fuera de GAM o No dijo. NUNCA la dirección." sqref="F2:F301" xr:uid="{00000000-0002-0000-0200-000004000000}">
@@ -8406,10 +8591,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
@@ -8420,96 +8605,96 @@
   <sheetData>
     <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="25" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="B4" s="26"/>
       <c r="C4" s="2" t="s">
-        <v>113</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="25" t="s">
-        <v>114</v>
+        <v>133</v>
       </c>
       <c r="B5" s="26"/>
       <c r="C5" s="2" t="s">
-        <v>115</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="B6" s="55" t="str">
-        <f>IF(SUM(I79:I85)=0,"Sin inconsistencias detectadas en «Consultas».","Hay "&amp;SUM(I79:I85)&amp;" inconsistencias: revisá las filas en rojo de «Consultas» y el control al final de esta hoja.")</f>
+        <v>135</v>
+      </c>
+      <c r="B6" s="59" t="str">
+        <f>IF(SUM(I98:I105)=0,"Sin inconsistencias detectadas en «Consultas».","Hay "&amp;SUM(I98:I105)&amp;" inconsistencias: revisá las filas en rojo de «Consultas» y el control al final de esta hoja.")</f>
         <v>Sin inconsistencias detectadas en «Consultas».</v>
       </c>
-      <c r="C6" s="56"/>
-      <c r="D6" s="56"/>
-      <c r="E6" s="56"/>
-      <c r="F6" s="56"/>
-      <c r="G6" s="56"/>
-      <c r="H6" s="56"/>
-      <c r="I6" s="56"/>
-      <c r="J6" s="56"/>
-      <c r="K6" s="56"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="58"/>
+      <c r="J6" s="58"/>
+      <c r="K6" s="58"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>117</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>68</v>
+        <v>87</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>120</v>
+        <v>139</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>121</v>
+        <v>140</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>122</v>
+        <v>141</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>123</v>
+        <v>142</v>
       </c>
       <c r="H9" s="27" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>125</v>
+        <v>144</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>127</v>
+        <v>146</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>55</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="28" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="B10" s="29">
         <f>COUNTIFS(Consultas!$D$2:$D$1000,$A10,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
@@ -8555,7 +8740,7 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="28" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B11" s="29">
         <f>COUNTIFS(Consultas!$D$2:$D$1000,$A11,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
@@ -8693,7 +8878,7 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="28" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B14" s="29">
         <f>COUNTIFS(Consultas!$D$2:$D$1000,$A14,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
@@ -8720,7 +8905,7 @@
         <v>0</v>
       </c>
       <c r="H14" s="35" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="I14" s="32" t="str">
         <f t="shared" si="0"/>
@@ -8735,12 +8920,12 @@
         <v>NO CALCULABLE</v>
       </c>
       <c r="L14" s="35" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="28" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B15" s="29">
         <f>COUNTIFS(Consultas!$D$2:$D$1000,$A15,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
@@ -8767,7 +8952,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="35" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
       <c r="I15" s="32" t="str">
         <f t="shared" si="0"/>
@@ -8782,12 +8967,12 @@
         <v>NO CALCULABLE</v>
       </c>
       <c r="L15" s="35" t="s">
-        <v>130</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="36" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="B16" s="37">
         <f t="shared" ref="B16:G16" si="3">SUM(B10:B15)</f>
@@ -8834,64 +9019,64 @@
         <v>NO CALCULABLE</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>139</v>
+        <v>158</v>
       </c>
       <c r="B25" s="27" t="s">
-        <v>140</v>
+        <v>159</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>141</v>
+        <v>160</v>
       </c>
       <c r="D25" s="27" t="s">
-        <v>142</v>
+        <v>161</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>131</v>
+        <v>150</v>
       </c>
       <c r="F25" s="27" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="28" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="B26" s="42"/>
       <c r="C26" s="42"/>
@@ -8902,9 +9087,9 @@
       </c>
       <c r="F26" s="26"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="28" t="s">
-        <v>129</v>
+        <v>148</v>
       </c>
       <c r="B27" s="42"/>
       <c r="C27" s="42"/>
@@ -8915,7 +9100,7 @@
       </c>
       <c r="F27" s="26"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="28" t="s">
         <v>19</v>
       </c>
@@ -8928,7 +9113,7 @@
       </c>
       <c r="F28" s="26"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="28" t="s">
         <v>21</v>
       </c>
@@ -8941,1021 +9126,1604 @@
       </c>
       <c r="F29" s="26"/>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="H35" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="I35" s="9" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A32" s="57" t="s">
+      <c r="J35" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="B32" s="52"/>
-      <c r="C32" s="52"/>
-      <c r="D32" s="52"/>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="52"/>
-      <c r="H32" s="52"/>
-      <c r="I32" s="44"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="57" t="s">
+      <c r="K35" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="B33" s="52"/>
-      <c r="C33" s="52"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="52"/>
-      <c r="F33" s="52"/>
-      <c r="G33" s="52"/>
-      <c r="H33" s="52"/>
-      <c r="I33" s="44"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="57" t="s">
-        <v>147</v>
-      </c>
-      <c r="B34" s="52"/>
-      <c r="C34" s="52"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="52"/>
-      <c r="H34" s="52"/>
-      <c r="I34" s="44"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="57" t="s">
-        <v>148</v>
-      </c>
-      <c r="B35" s="52"/>
-      <c r="C35" s="52"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="52"/>
-      <c r="H35" s="52"/>
-      <c r="I35" s="44"/>
-    </row>
-    <row r="36" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="25" t="s">
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="28" t="s">
+        <v>159</v>
+      </c>
+      <c r="B36" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A36,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C36" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A36,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A36,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E36" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A36,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F36" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A36,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G36" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A36,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="35" t="s">
         <v>149</v>
       </c>
-      <c r="B36" s="55" t="str">
-        <f>IF(COUNTA($I$32,$I$33,$I$34,$I$35)&lt;4,"Contestá las cuatro preguntas antes de comparar piezas.",IF(OR($I$32="Sí",$I$33="Sí",$I$34="No",$I$35="No"),"Comparación entre piezas NO VÁLIDA en este periodo: extendé o repetí la prueba con condiciones parejas.","Condiciones parejas declaradas. Con pocas consultas igual no se declara ganador: seguí observando."))</f>
-        <v>Contestá las cuatro preguntas antes de comparar piezas.</v>
-      </c>
-      <c r="C36" s="56"/>
-      <c r="D36" s="56"/>
-      <c r="E36" s="56"/>
-      <c r="F36" s="56"/>
-      <c r="G36" s="56"/>
-      <c r="H36" s="56"/>
-      <c r="I36" s="56"/>
-      <c r="J36" s="56"/>
-      <c r="K36" s="56"/>
+      <c r="I36" s="32" t="str">
+        <f t="shared" ref="I36:I46" si="4">IF(B36=0,"NO CALCULABLE",C36/B36)</f>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J36" s="32" t="str">
+        <f t="shared" ref="J36:J46" si="5">IF(C36=0,"NO CALCULABLE",E36/C36)</f>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K36" s="35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="B37" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A37,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C37" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A37,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D37" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A37,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E37" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A37,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F37" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A37,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A37,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I37" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J37" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K37" s="35" t="s">
+        <v>149</v>
+      </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>150</v>
+      <c r="A38" s="28" t="s">
+        <v>36</v>
+      </c>
+      <c r="B38" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A38,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A38,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A38,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A38,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F38" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A38,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G38" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A38,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I38" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J38" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K38" s="35" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="2" t="s">
-        <v>151</v>
+      <c r="A39" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A39,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C39" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A39,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D39" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A39,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E39" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A39,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F39" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A39,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G39" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A39,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I39" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J39" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K39" s="35" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="9" t="s">
-        <v>139</v>
-      </c>
-      <c r="B41" s="27" t="s">
-        <v>153</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>154</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="F41" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="G41" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="H41" s="9" t="s">
-        <v>125</v>
-      </c>
-      <c r="I41" s="9" t="s">
-        <v>126</v>
-      </c>
-      <c r="J41" s="27" t="s">
-        <v>155</v>
-      </c>
-      <c r="K41" s="9" t="s">
-        <v>55</v>
+      <c r="A40" s="28" t="s">
+        <v>161</v>
+      </c>
+      <c r="B40" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A40,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C40" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A40,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D40" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A40,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E40" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A40,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F40" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A40,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G40" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A40,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I40" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J40" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K40" s="35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A41,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C41" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A41,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D41" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A41,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E41" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A41,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F41" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A41,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A41,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I41" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J41" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K41" s="35" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="28" t="s">
-        <v>128</v>
-      </c>
-      <c r="B42" s="26"/>
-      <c r="C42" s="45" t="str">
-        <f>IF($B42="","Falta fecha",$B42+3)</f>
-        <v>Falta fecha</v>
-      </c>
-      <c r="D42" s="29" t="str">
-        <f>IF($B42="","",COUNTIFS(Consultas!$D$2:$D$1000,$A42,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B42,Consultas!$B$2:$B$1000,"&lt;="&amp;($B42+3)))</f>
-        <v/>
-      </c>
-      <c r="E42" s="29" t="str">
-        <f>IF($B42="","",COUNTIFS(Consultas!$D$2:$D$1000,$A42,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B42,Consultas!$B$2:$B$1000,"&lt;="&amp;($B42+3),Consultas!$H$2:$H$1000,"Sí"))</f>
-        <v/>
-      </c>
-      <c r="F42" s="29" t="str">
-        <f>IF($B42="","",COUNTIFS(Consultas!$D$2:$D$1000,$A42,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B42,Consultas!$B$2:$B$1000,"&lt;="&amp;($B42+3),Consultas!$I$2:$I$1000,"Sí"))</f>
-        <v/>
-      </c>
-      <c r="G42" s="29" t="str">
-        <f>IF($B42="","",COUNTIFS(Consultas!$D$2:$D$1000,$A42,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B42,Consultas!$B$2:$B$1000,"&lt;="&amp;($B42+3),Consultas!$J$2:$J$1000,"Sí"))</f>
-        <v/>
-      </c>
-      <c r="H42" s="32" t="str">
-        <f>IF(N(D42)=0,"NO CALCULABLE",E42/D42)</f>
+        <v>42</v>
+      </c>
+      <c r="B42" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A42,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C42" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A42,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D42" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A42,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E42" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A42,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F42" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A42,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G42" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A42,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="31"/>
+      <c r="I42" s="32" t="str">
+        <f t="shared" si="4"/>
         <v>NO CALCULABLE</v>
       </c>
-      <c r="I42" s="32" t="str">
-        <f>IF(N(E42)=0,"NO CALCULABLE",G42/E42)</f>
+      <c r="J42" s="32" t="str">
+        <f t="shared" si="5"/>
         <v>NO CALCULABLE</v>
       </c>
-      <c r="J42" s="42"/>
-      <c r="K42" s="34" t="str">
-        <f>IF(OR($B42="",N(J42)=0),"NO CALCULABLE",E42/J42)</f>
+      <c r="K42" s="33" t="str">
+        <f>IF(C42=0,"NO CALCULABLE",IF(N(H42)&lt;=0,"SIN PAUTA",H42/C42))</f>
         <v>NO CALCULABLE</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" s="28" t="s">
-        <v>129</v>
-      </c>
-      <c r="B43" s="26"/>
-      <c r="C43" s="45" t="str">
-        <f>IF($B43="","Falta fecha",$B43+3)</f>
+        <v>167</v>
+      </c>
+      <c r="B43" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A43,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C43" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A43,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A43,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E43" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A43,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F43" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A43,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G43" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A43,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I43" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J43" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K43" s="35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B44" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A44,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C44" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A44,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D44" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A44,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E44" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A44,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F44" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A44,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G44" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A44,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I44" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J44" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K44" s="35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="B45" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A45,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5))</f>
+        <v>0</v>
+      </c>
+      <c r="C45" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A45,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$H$2:$H$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="D45" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A45,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$I$2:$I$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="E45" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A45,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$J$2:$J$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="F45" s="29">
+        <f>COUNTIFS(Consultas!$C$2:$C$1000,$A45,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="G45" s="30">
+        <f>SUMIFS(Consultas!$L$2:$L$1000,Consultas!$C$2:$C$1000,$A45,Consultas!$D$2:$D$1000,"&lt;&gt;",Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$K$2:$K$1000,"Sí")</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="35" t="s">
+        <v>149</v>
+      </c>
+      <c r="I45" s="32" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J45" s="32" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K45" s="35" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B46" s="37">
+        <f t="shared" ref="B46:G46" si="6">SUM(B36:B45)</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="37">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="D46" s="37">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="E46" s="37">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="F46" s="37">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="G46" s="38">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H46" s="44" t="s">
+        <v>149</v>
+      </c>
+      <c r="I46" s="40" t="str">
+        <f t="shared" si="4"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J46" s="40" t="str">
+        <f t="shared" si="5"/>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="K46" s="44" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" s="56" t="s">
+        <v>170</v>
+      </c>
+      <c r="B47" s="53"/>
+      <c r="C47" s="53"/>
+      <c r="D47" s="53"/>
+      <c r="E47" s="53"/>
+      <c r="F47" s="53"/>
+      <c r="G47" s="53"/>
+      <c r="H47" s="53"/>
+      <c r="I47" s="45">
+        <f>$B$16-B46</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" s="57" t="str">
+        <f>IF(AND(SUMIF($H$10:$H$13,"&gt;0")&gt;0,N($H$42)&gt;0),"Hay pauta escrita en los dos cuadros: confirmá que son anuncios distintos y que ningún gasto está anotado dos veces.","")</f>
+        <v/>
+      </c>
+      <c r="B48" s="58"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="58"/>
+      <c r="G48" s="58"/>
+      <c r="H48" s="58"/>
+      <c r="I48" s="58"/>
+      <c r="J48" s="58"/>
+      <c r="K48" s="58"/>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" s="56" t="s">
+        <v>172</v>
+      </c>
+      <c r="B51" s="53"/>
+      <c r="C51" s="53"/>
+      <c r="D51" s="53"/>
+      <c r="E51" s="53"/>
+      <c r="F51" s="53"/>
+      <c r="G51" s="53"/>
+      <c r="H51" s="53"/>
+      <c r="I51" s="46"/>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="56" t="s">
+        <v>173</v>
+      </c>
+      <c r="B52" s="53"/>
+      <c r="C52" s="53"/>
+      <c r="D52" s="53"/>
+      <c r="E52" s="53"/>
+      <c r="F52" s="53"/>
+      <c r="G52" s="53"/>
+      <c r="H52" s="53"/>
+      <c r="I52" s="46"/>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="56" t="s">
+        <v>174</v>
+      </c>
+      <c r="B53" s="53"/>
+      <c r="C53" s="53"/>
+      <c r="D53" s="53"/>
+      <c r="E53" s="53"/>
+      <c r="F53" s="53"/>
+      <c r="G53" s="53"/>
+      <c r="H53" s="53"/>
+      <c r="I53" s="46"/>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="56" t="s">
+        <v>175</v>
+      </c>
+      <c r="B54" s="53"/>
+      <c r="C54" s="53"/>
+      <c r="D54" s="53"/>
+      <c r="E54" s="53"/>
+      <c r="F54" s="53"/>
+      <c r="G54" s="53"/>
+      <c r="H54" s="53"/>
+      <c r="I54" s="46"/>
+    </row>
+    <row r="55" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B55" s="59" t="str">
+        <f>IF(COUNTA($I$51,$I$52,$I$53,$I$54)&lt;4,"Contestá las cuatro preguntas antes de comparar piezas.",IF(OR($I$51="Sí",$I$52="Sí",$I$53="No",$I$54="No"),"Comparación entre piezas NO VÁLIDA en este periodo: extendé o repetí la prueba con condiciones parejas.","Condiciones parejas declaradas. Con pocas consultas igual no se declara ganador: seguí observando."))</f>
+        <v>Contestá las cuatro preguntas antes de comparar piezas.</v>
+      </c>
+      <c r="C55" s="58"/>
+      <c r="D55" s="58"/>
+      <c r="E55" s="58"/>
+      <c r="F55" s="58"/>
+      <c r="G55" s="58"/>
+      <c r="H55" s="58"/>
+      <c r="I55" s="58"/>
+      <c r="J55" s="58"/>
+      <c r="K55" s="58"/>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B60" s="27" t="s">
+        <v>180</v>
+      </c>
+      <c r="C60" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="E60" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="H60" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="I60" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="J60" s="27" t="s">
+        <v>182</v>
+      </c>
+      <c r="K60" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B61" s="26"/>
+      <c r="C61" s="47" t="str">
+        <f>IF($B61="","Falta fecha",$B61+3)</f>
         <v>Falta fecha</v>
       </c>
-      <c r="D43" s="29" t="str">
-        <f>IF($B43="","",COUNTIFS(Consultas!$D$2:$D$1000,$A43,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B43,Consultas!$B$2:$B$1000,"&lt;="&amp;($B43+3)))</f>
-        <v/>
-      </c>
-      <c r="E43" s="29" t="str">
-        <f>IF($B43="","",COUNTIFS(Consultas!$D$2:$D$1000,$A43,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B43,Consultas!$B$2:$B$1000,"&lt;="&amp;($B43+3),Consultas!$H$2:$H$1000,"Sí"))</f>
-        <v/>
-      </c>
-      <c r="F43" s="29" t="str">
-        <f>IF($B43="","",COUNTIFS(Consultas!$D$2:$D$1000,$A43,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B43,Consultas!$B$2:$B$1000,"&lt;="&amp;($B43+3),Consultas!$I$2:$I$1000,"Sí"))</f>
-        <v/>
-      </c>
-      <c r="G43" s="29" t="str">
-        <f>IF($B43="","",COUNTIFS(Consultas!$D$2:$D$1000,$A43,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B43,Consultas!$B$2:$B$1000,"&lt;="&amp;($B43+3),Consultas!$J$2:$J$1000,"Sí"))</f>
-        <v/>
-      </c>
-      <c r="H43" s="32" t="str">
-        <f>IF(N(D43)=0,"NO CALCULABLE",E43/D43)</f>
+      <c r="D61" s="29" t="str">
+        <f>IF($B61="","",COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B61,Consultas!$B$2:$B$1000,"&lt;="&amp;($B61+3)))</f>
+        <v/>
+      </c>
+      <c r="E61" s="29" t="str">
+        <f>IF($B61="","",COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B61,Consultas!$B$2:$B$1000,"&lt;="&amp;($B61+3),Consultas!$H$2:$H$1000,"Sí"))</f>
+        <v/>
+      </c>
+      <c r="F61" s="29" t="str">
+        <f>IF($B61="","",COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B61,Consultas!$B$2:$B$1000,"&lt;="&amp;($B61+3),Consultas!$I$2:$I$1000,"Sí"))</f>
+        <v/>
+      </c>
+      <c r="G61" s="29" t="str">
+        <f>IF($B61="","",COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B61,Consultas!$B$2:$B$1000,"&lt;="&amp;($B61+3),Consultas!$J$2:$J$1000,"Sí"))</f>
+        <v/>
+      </c>
+      <c r="H61" s="32" t="str">
+        <f>IF(N(D61)=0,"NO CALCULABLE",E61/D61)</f>
         <v>NO CALCULABLE</v>
       </c>
-      <c r="I43" s="32" t="str">
-        <f>IF(N(E43)=0,"NO CALCULABLE",G43/E43)</f>
+      <c r="I61" s="32" t="str">
+        <f>IF(N(E61)=0,"NO CALCULABLE",G61/E61)</f>
         <v>NO CALCULABLE</v>
       </c>
-      <c r="J43" s="42"/>
-      <c r="K43" s="34" t="str">
-        <f>IF(OR($B43="",N(J43)=0),"NO CALCULABLE",E43/J43)</f>
+      <c r="J61" s="42"/>
+      <c r="K61" s="34" t="str">
+        <f>IF(OR($B61="",N(J61)=0),"NO CALCULABLE",E61/J61)</f>
         <v>NO CALCULABLE</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="B44" s="46"/>
-      <c r="C44" s="46"/>
-      <c r="D44" s="47" t="str">
-        <f>IF(OR($B$42="",$B$43=""),"",D43-D42)</f>
-        <v/>
-      </c>
-      <c r="E44" s="47" t="str">
-        <f>IF(OR($B$42="",$B$43=""),"",E43-E42)</f>
-        <v/>
-      </c>
-      <c r="F44" s="47" t="str">
-        <f>IF(OR($B$42="",$B$43=""),"",F43-F42)</f>
-        <v/>
-      </c>
-      <c r="G44" s="47" t="str">
-        <f>IF(OR($B$42="",$B$43=""),"",G43-G42)</f>
-        <v/>
-      </c>
-      <c r="H44" s="46"/>
-      <c r="I44" s="46"/>
-      <c r="J44" s="46"/>
-      <c r="K44" s="46"/>
-    </row>
-    <row r="45" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="25" t="s">
-        <v>149</v>
-      </c>
-      <c r="B45" s="55" t="str">
-        <f>IF(OR($B$42="",$B$43=""),"Escribí las dos fechas de publicación para comparar.",IF(COUNTA($I$32,$I$33,$I$34,$I$35)&lt;4,"Contestá las cuatro preguntas de condiciones antes de comparar.",IF(OR($I$32="Sí",$I$33="Sí",$I$34="No",$I$35="No"),"Comparación NO VÁLIDA: las condiciones no fueron parejas. Repetí la prueba.",IF($E$44=0,"GAME1 y GAME2 tuvieron las mismas consultas cualificadas.","GAME2 tuvo "&amp;ABS($E$44)&amp;" consulta(s) cualificada(s) "&amp;IF($E$44&gt;0,"más","menos")&amp;" que GAME1.")&amp;IF(OR(N($J$42)=0,N($J$43)=0)," Falta el alcance de al menos una pieza: la lectura es solo descriptiva y se comparan volúmenes absolutos junto al alcance conocido."," Las dos piezas tienen alcance: mirá también Cualificadas / alcance.")&amp;" Es una señal exploratoria, no un ganador: no se sabe en qué dirección influyen el día, el orden ni el alcance.")))</f>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="28" t="s">
+        <v>148</v>
+      </c>
+      <c r="B62" s="26"/>
+      <c r="C62" s="47" t="str">
+        <f>IF($B62="","Falta fecha",$B62+3)</f>
+        <v>Falta fecha</v>
+      </c>
+      <c r="D62" s="29" t="str">
+        <f>IF($B62="","",COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B62,Consultas!$B$2:$B$1000,"&lt;="&amp;($B62+3)))</f>
+        <v/>
+      </c>
+      <c r="E62" s="29" t="str">
+        <f>IF($B62="","",COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B62,Consultas!$B$2:$B$1000,"&lt;="&amp;($B62+3),Consultas!$H$2:$H$1000,"Sí"))</f>
+        <v/>
+      </c>
+      <c r="F62" s="29" t="str">
+        <f>IF($B62="","",COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B62,Consultas!$B$2:$B$1000,"&lt;="&amp;($B62+3),Consultas!$I$2:$I$1000,"Sí"))</f>
+        <v/>
+      </c>
+      <c r="G62" s="29" t="str">
+        <f>IF($B62="","",COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;$B62,Consultas!$B$2:$B$1000,"&lt;="&amp;($B62+3),Consultas!$J$2:$J$1000,"Sí"))</f>
+        <v/>
+      </c>
+      <c r="H62" s="32" t="str">
+        <f>IF(N(D62)=0,"NO CALCULABLE",E62/D62)</f>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="I62" s="32" t="str">
+        <f>IF(N(E62)=0,"NO CALCULABLE",G62/E62)</f>
+        <v>NO CALCULABLE</v>
+      </c>
+      <c r="J62" s="42"/>
+      <c r="K62" s="34" t="str">
+        <f>IF(OR($B62="",N(J62)=0),"NO CALCULABLE",E62/J62)</f>
+        <v>NO CALCULABLE</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="36" t="s">
+        <v>183</v>
+      </c>
+      <c r="B63" s="48"/>
+      <c r="C63" s="48"/>
+      <c r="D63" s="49" t="str">
+        <f>IF(OR($B$61="",$B$62=""),"",D62-D61)</f>
+        <v/>
+      </c>
+      <c r="E63" s="49" t="str">
+        <f>IF(OR($B$61="",$B$62=""),"",E62-E61)</f>
+        <v/>
+      </c>
+      <c r="F63" s="49" t="str">
+        <f>IF(OR($B$61="",$B$62=""),"",F62-F61)</f>
+        <v/>
+      </c>
+      <c r="G63" s="49" t="str">
+        <f>IF(OR($B$61="",$B$62=""),"",G62-G61)</f>
+        <v/>
+      </c>
+      <c r="H63" s="48"/>
+      <c r="I63" s="48"/>
+      <c r="J63" s="48"/>
+      <c r="K63" s="48"/>
+    </row>
+    <row r="64" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="25" t="s">
+        <v>176</v>
+      </c>
+      <c r="B64" s="59" t="str">
+        <f>IF(OR($B$61="",$B$62=""),"Escribí las dos fechas de publicación para comparar.",IF(COUNTA($I$51,$I$52,$I$53,$I$54)&lt;4,"Contestá las cuatro preguntas de condiciones antes de comparar.",IF(OR($I$51="Sí",$I$52="Sí",$I$53="No",$I$54="No"),"Comparación NO VÁLIDA: las condiciones no fueron parejas. Repetí la prueba.",IF($E$63=0,"GAME1 y GAME2 tuvieron las mismas consultas cualificadas.","GAME2 tuvo "&amp;ABS($E$63)&amp;" consulta(s) cualificada(s) "&amp;IF($E$63&gt;0,"más","menos")&amp;" que GAME1.")&amp;IF(OR(N($J$61)=0,N($J$62)=0)," Falta el alcance de al menos una pieza: la lectura es solo descriptiva y se comparan volúmenes absolutos junto al alcance conocido."," Las dos piezas tienen alcance: mirá también Cualificadas / alcance.")&amp;" Es una señal exploratoria, no un ganador: no se sabe en qué dirección influyen el día, el orden ni el alcance.")))</f>
         <v>Escribí las dos fechas de publicación para comparar.</v>
       </c>
-      <c r="C45" s="56"/>
-      <c r="D45" s="56"/>
-      <c r="E45" s="56"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="56"/>
-      <c r="H45" s="56"/>
-      <c r="I45" s="56"/>
-      <c r="J45" s="56"/>
-      <c r="K45" s="56"/>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B48" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="D48" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="28" t="s">
-        <v>128</v>
-      </c>
-      <c r="B49" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A49,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="C49" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A49,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="D49" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A49,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
-        <v>0</v>
-      </c>
-      <c r="E49" s="29">
-        <f>$B$10-SUM(B49:D49)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="28" t="s">
-        <v>129</v>
-      </c>
-      <c r="B50" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A50,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="C50" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A50,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="D50" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A50,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
-        <v>0</v>
-      </c>
-      <c r="E50" s="29">
-        <f>$B$11-SUM(B50:D50)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B51" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A51,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="C51" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A51,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A51,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
-        <v>0</v>
-      </c>
-      <c r="E51" s="29">
-        <f>$B$12-SUM(B51:D51)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="B52" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A52,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="C52" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A52,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="D52" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A52,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
-        <v>0</v>
-      </c>
-      <c r="E52" s="29">
-        <f>$B$13-SUM(B52:D52)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="B53" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A53,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="C53" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A53,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="D53" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A53,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
-        <v>0</v>
-      </c>
-      <c r="E53" s="29">
-        <f>$B$14-SUM(B53:D53)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A54" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B54" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A54,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="C54" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A54,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
-        <v>0</v>
-      </c>
-      <c r="D54" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A54,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
-        <v>0</v>
-      </c>
-      <c r="E54" s="29">
-        <f>$B$15-SUM(B54:D54)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="36" t="s">
-        <v>131</v>
-      </c>
-      <c r="B55" s="37">
-        <f>SUM(B49:B54)</f>
-        <v>0</v>
-      </c>
-      <c r="C55" s="37">
-        <f>SUM(C49:C54)</f>
-        <v>0</v>
-      </c>
-      <c r="D55" s="37">
-        <f>SUM(D49:D54)</f>
-        <v>0</v>
-      </c>
-      <c r="E55" s="37">
-        <f>SUM(E49:E54)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A57" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B58" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="C58" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="D58" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="E58" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="F58" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="G58" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="H58" s="9" t="s">
+      <c r="C64" s="58"/>
+      <c r="D64" s="58"/>
+      <c r="E64" s="58"/>
+      <c r="F64" s="58"/>
+      <c r="G64" s="58"/>
+      <c r="H64" s="58"/>
+      <c r="I64" s="58"/>
+      <c r="J64" s="58"/>
+      <c r="K64" s="58"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="3" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A67" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B67" s="9" t="s">
+        <v>185</v>
+      </c>
+      <c r="C67" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="D67" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="I58" s="9" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="28" t="s">
-        <v>128</v>
-      </c>
-      <c r="B59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
-        <v>0</v>
-      </c>
-      <c r="C59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
-        <v>0</v>
-      </c>
-      <c r="D59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
-        <v>0</v>
-      </c>
-      <c r="E59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
-        <v>0</v>
-      </c>
-      <c r="F59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
-        <v>0</v>
-      </c>
-      <c r="G59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
-        <v>0</v>
-      </c>
-      <c r="H59" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A59,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
-        <v>0</v>
-      </c>
-      <c r="I59" s="29">
-        <f>$B$10-SUM(B59:H59)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="28" t="s">
-        <v>129</v>
-      </c>
-      <c r="B60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
-        <v>0</v>
-      </c>
-      <c r="C60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
-        <v>0</v>
-      </c>
-      <c r="D60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
-        <v>0</v>
-      </c>
-      <c r="E60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
-        <v>0</v>
-      </c>
-      <c r="F60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
-        <v>0</v>
-      </c>
-      <c r="G60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
-        <v>0</v>
-      </c>
-      <c r="H60" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A60,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
-        <v>0</v>
-      </c>
-      <c r="I60" s="29">
-        <f>$B$11-SUM(B60:H60)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="B61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
-        <v>0</v>
-      </c>
-      <c r="C61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
-        <v>0</v>
-      </c>
-      <c r="D61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
-        <v>0</v>
-      </c>
-      <c r="E61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
-        <v>0</v>
-      </c>
-      <c r="F61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
-        <v>0</v>
-      </c>
-      <c r="G61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
-        <v>0</v>
-      </c>
-      <c r="H61" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A61,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
-        <v>0</v>
-      </c>
-      <c r="I61" s="29">
-        <f>$B$12-SUM(B61:H61)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="28" t="s">
-        <v>21</v>
-      </c>
-      <c r="B62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
-        <v>0</v>
-      </c>
-      <c r="C62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
-        <v>0</v>
-      </c>
-      <c r="D62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
-        <v>0</v>
-      </c>
-      <c r="E62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
-        <v>0</v>
-      </c>
-      <c r="F62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
-        <v>0</v>
-      </c>
-      <c r="G62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
-        <v>0</v>
-      </c>
-      <c r="H62" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A62,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
-        <v>0</v>
-      </c>
-      <c r="I62" s="29">
-        <f>$B$13-SUM(B62:H62)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="28" t="s">
-        <v>23</v>
-      </c>
-      <c r="B63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
-        <v>0</v>
-      </c>
-      <c r="C63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
-        <v>0</v>
-      </c>
-      <c r="D63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
-        <v>0</v>
-      </c>
-      <c r="E63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
-        <v>0</v>
-      </c>
-      <c r="F63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
-        <v>0</v>
-      </c>
-      <c r="G63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
-        <v>0</v>
-      </c>
-      <c r="H63" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A63,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
-        <v>0</v>
-      </c>
-      <c r="I63" s="29">
-        <f>$B$14-SUM(B63:H63)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="28" t="s">
-        <v>25</v>
-      </c>
-      <c r="B64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
-        <v>0</v>
-      </c>
-      <c r="C64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
-        <v>0</v>
-      </c>
-      <c r="D64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
-        <v>0</v>
-      </c>
-      <c r="E64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
-        <v>0</v>
-      </c>
-      <c r="F64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
-        <v>0</v>
-      </c>
-      <c r="G64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
-        <v>0</v>
-      </c>
-      <c r="H64" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A64,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
-        <v>0</v>
-      </c>
-      <c r="I64" s="29">
-        <f>$B$15-SUM(B64:H64)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" s="36" t="s">
-        <v>131</v>
-      </c>
-      <c r="B65" s="37">
-        <f t="shared" ref="B65:I65" si="4">SUM(B59:B64)</f>
-        <v>0</v>
-      </c>
-      <c r="C65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="D65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="E65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="F65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="G65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="H65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="I65" s="37">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A67" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="B68" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="C68" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="D68" s="9" t="s">
-        <v>174</v>
+      <c r="E67" s="9" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B68" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A68,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A68,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A68,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
+        <v>0</v>
+      </c>
+      <c r="E68" s="29">
+        <f>$B$10-SUM(B68:D68)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="28" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="B69" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A69,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A69,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
         <v>0</v>
       </c>
       <c r="C69" s="29">
-        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A69,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="D69" s="48" t="str">
-        <f t="shared" ref="D69:D75" si="5">IF(B69=0,"NO CALCULABLE",C69/B69)</f>
-        <v>NO CALCULABLE</v>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A69,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A69,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
+        <v>0</v>
+      </c>
+      <c r="E69" s="29">
+        <f>$B$11-SUM(B69:D69)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="28" t="s">
-        <v>129</v>
+        <v>19</v>
       </c>
       <c r="B70" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A70,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A70,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
         <v>0</v>
       </c>
       <c r="C70" s="29">
-        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A70,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="D70" s="48" t="str">
-        <f t="shared" si="5"/>
-        <v>NO CALCULABLE</v>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A70,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A70,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
+        <v>0</v>
+      </c>
+      <c r="E70" s="29">
+        <f>$B$12-SUM(B70:D70)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="28" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B71" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A71,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A71,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
         <v>0</v>
       </c>
       <c r="C71" s="29">
-        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A71,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="D71" s="48" t="str">
-        <f t="shared" si="5"/>
-        <v>NO CALCULABLE</v>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A71,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A71,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
+        <v>0</v>
+      </c>
+      <c r="E71" s="29">
+        <f>$B$13-SUM(B71:D71)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="28" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B72" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A72,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A72,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
         <v>0</v>
       </c>
       <c r="C72" s="29">
-        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A72,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="D72" s="48" t="str">
-        <f t="shared" si="5"/>
-        <v>NO CALCULABLE</v>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A72,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A72,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
+        <v>0</v>
+      </c>
+      <c r="E72" s="29">
+        <f>$B$14-SUM(B72:D72)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="28" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B73" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A73,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A73,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"GAM")</f>
         <v>0</v>
       </c>
       <c r="C73" s="29">
-        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A73,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="D73" s="48" t="str">
-        <f t="shared" si="5"/>
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A73,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"Fuera de GAM")</f>
+        <v>0</v>
+      </c>
+      <c r="D73" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A73,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$F$2:$F$1000,"No dijo")</f>
+        <v>0</v>
+      </c>
+      <c r="E73" s="29">
+        <f>$B$15-SUM(B73:D73)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A74" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B74" s="37">
+        <f>SUM(B68:B73)</f>
+        <v>0</v>
+      </c>
+      <c r="C74" s="37">
+        <f>SUM(C68:C73)</f>
+        <v>0</v>
+      </c>
+      <c r="D74" s="37">
+        <f>SUM(D68:D73)</f>
+        <v>0</v>
+      </c>
+      <c r="E74" s="37">
+        <f>SUM(E68:E73)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A77" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B77" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="D77" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="E77" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>193</v>
+      </c>
+      <c r="G77" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="H77" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="I77" s="9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
+        <v>0</v>
+      </c>
+      <c r="C78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
+        <v>0</v>
+      </c>
+      <c r="D78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
+        <v>0</v>
+      </c>
+      <c r="E78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
+        <v>0</v>
+      </c>
+      <c r="F78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
+        <v>0</v>
+      </c>
+      <c r="G78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
+        <v>0</v>
+      </c>
+      <c r="H78" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A78,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
+        <v>0</v>
+      </c>
+      <c r="I78" s="29">
+        <f>$B$10-SUM(B78:H78)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A79" s="28" t="s">
+        <v>148</v>
+      </c>
+      <c r="B79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
+        <v>0</v>
+      </c>
+      <c r="C79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
+        <v>0</v>
+      </c>
+      <c r="D79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
+        <v>0</v>
+      </c>
+      <c r="E79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
+        <v>0</v>
+      </c>
+      <c r="F79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
+        <v>0</v>
+      </c>
+      <c r="G79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
+        <v>0</v>
+      </c>
+      <c r="H79" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A79,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
+        <v>0</v>
+      </c>
+      <c r="I79" s="29">
+        <f>$B$11-SUM(B79:H79)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A80" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
+        <v>0</v>
+      </c>
+      <c r="C80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
+        <v>0</v>
+      </c>
+      <c r="G80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
+        <v>0</v>
+      </c>
+      <c r="H80" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A80,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
+        <v>0</v>
+      </c>
+      <c r="I80" s="29">
+        <f>$B$12-SUM(B80:H80)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A81" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
+        <v>0</v>
+      </c>
+      <c r="C81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
+        <v>0</v>
+      </c>
+      <c r="D81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
+        <v>0</v>
+      </c>
+      <c r="E81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
+        <v>0</v>
+      </c>
+      <c r="G81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
+        <v>0</v>
+      </c>
+      <c r="H81" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A81,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
+        <v>0</v>
+      </c>
+      <c r="I81" s="29">
+        <f>$B$13-SUM(B81:H81)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A82" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
+        <v>0</v>
+      </c>
+      <c r="C82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
+        <v>0</v>
+      </c>
+      <c r="D82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
+        <v>0</v>
+      </c>
+      <c r="E82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
+        <v>0</v>
+      </c>
+      <c r="F82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
+        <v>0</v>
+      </c>
+      <c r="G82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
+        <v>0</v>
+      </c>
+      <c r="H82" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A82,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
+        <v>0</v>
+      </c>
+      <c r="I82" s="29">
+        <f>$B$14-SUM(B82:H82)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A83" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Precio")</f>
+        <v>0</v>
+      </c>
+      <c r="C83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Compatibilidad")</f>
+        <v>0</v>
+      </c>
+      <c r="D83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Envío")</f>
+        <v>0</v>
+      </c>
+      <c r="E83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Garantía")</f>
+        <v>0</v>
+      </c>
+      <c r="F83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Confianza")</f>
+        <v>0</v>
+      </c>
+      <c r="G83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Stock")</f>
+        <v>0</v>
+      </c>
+      <c r="H83" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A83,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$N$2:$N$1000,"Otra")</f>
+        <v>0</v>
+      </c>
+      <c r="I83" s="29">
+        <f>$B$15-SUM(B83:H83)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A84" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B84" s="37">
+        <f t="shared" ref="B84:I84" si="7">SUM(B78:B83)</f>
+        <v>0</v>
+      </c>
+      <c r="C84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="D84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="E84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="F84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="G84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="H84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="I84" s="37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A87" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B87" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="C87" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" s="28" t="s">
+        <v>147</v>
+      </c>
+      <c r="B88" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A88,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="C88" s="29">
+        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A88,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D88" s="50" t="str">
+        <f t="shared" ref="D88:D94" si="8">IF(B88=0,"NO CALCULABLE",C88/B88)</f>
         <v>NO CALCULABLE</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A74" s="28" t="s">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" s="28" t="s">
+        <v>148</v>
+      </c>
+      <c r="B89" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A89,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="C89" s="29">
+        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A89,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D89" s="50" t="str">
+        <f t="shared" si="8"/>
+        <v>NO CALCULABLE</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" s="28" t="s">
+        <v>19</v>
+      </c>
+      <c r="B90" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A90,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="C90" s="29">
+        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A90,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D90" s="50" t="str">
+        <f t="shared" si="8"/>
+        <v>NO CALCULABLE</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" s="28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B91" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A91,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="C91" s="29">
+        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A91,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D91" s="50" t="str">
+        <f t="shared" si="8"/>
+        <v>NO CALCULABLE</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B74" s="29">
-        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A74,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="C74" s="29">
-        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A74,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
-        <v>0</v>
-      </c>
-      <c r="D74" s="48" t="str">
-        <f t="shared" si="5"/>
+      <c r="B92" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A92,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="C92" s="29">
+        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A92,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D92" s="50" t="str">
+        <f t="shared" si="8"/>
         <v>NO CALCULABLE</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A75" s="36" t="s">
-        <v>131</v>
-      </c>
-      <c r="B75" s="37">
-        <f>SUM(B69:B74)</f>
-        <v>0</v>
-      </c>
-      <c r="C75" s="37">
-        <f>SUM(C69:C74)</f>
-        <v>0</v>
-      </c>
-      <c r="D75" s="49" t="str">
-        <f t="shared" si="5"/>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B93" s="29">
+        <f>COUNTIFS(Consultas!$D$2:$D$1000,$A93,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="C93" s="29">
+        <f>SUMIFS(Consultas!$M$2:$M$1000,Consultas!$D$2:$D$1000,$A93,Consultas!$G$2:$G$1000,"&lt;&gt;Sí",Consultas!$B$2:$B$1000,"&gt;="&amp;IF($B$4="",1,$B$4),Consultas!$B$2:$B$1000,"&lt;="&amp;IF($B$5="",2958465,$B$5),Consultas!$M$2:$M$1000,"&gt;=0")</f>
+        <v>0</v>
+      </c>
+      <c r="D93" s="50" t="str">
+        <f t="shared" si="8"/>
         <v>NO CALCULABLE</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A78" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A79" s="57" t="s">
-        <v>177</v>
-      </c>
-      <c r="B79" s="52"/>
-      <c r="C79" s="52"/>
-      <c r="D79" s="52"/>
-      <c r="E79" s="52"/>
-      <c r="F79" s="52"/>
-      <c r="G79" s="52"/>
-      <c r="H79" s="52"/>
-      <c r="I79" s="50">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" s="36" t="s">
+        <v>150</v>
+      </c>
+      <c r="B94" s="37">
+        <f>SUM(B88:B93)</f>
+        <v>0</v>
+      </c>
+      <c r="C94" s="37">
+        <f>SUM(C88:C93)</f>
+        <v>0</v>
+      </c>
+      <c r="D94" s="51" t="str">
+        <f t="shared" si="8"/>
+        <v>NO CALCULABLE</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" s="3" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" s="56" t="s">
+        <v>203</v>
+      </c>
+      <c r="B98" s="53"/>
+      <c r="C98" s="53"/>
+      <c r="D98" s="53"/>
+      <c r="E98" s="53"/>
+      <c r="F98" s="53"/>
+      <c r="G98" s="53"/>
+      <c r="H98" s="53"/>
+      <c r="I98" s="45">
         <f>SUMPRODUCT((LEN(Consultas!$B$2:$B$1000)&gt;0)*(LEN(Consultas!$D$2:$D$1000)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A80" s="57" t="s">
-        <v>178</v>
-      </c>
-      <c r="B80" s="52"/>
-      <c r="C80" s="52"/>
-      <c r="D80" s="52"/>
-      <c r="E80" s="52"/>
-      <c r="F80" s="52"/>
-      <c r="G80" s="52"/>
-      <c r="H80" s="52"/>
-      <c r="I80" s="50">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" s="56" t="s">
+        <v>204</v>
+      </c>
+      <c r="B99" s="53"/>
+      <c r="C99" s="53"/>
+      <c r="D99" s="53"/>
+      <c r="E99" s="53"/>
+      <c r="F99" s="53"/>
+      <c r="G99" s="53"/>
+      <c r="H99" s="53"/>
+      <c r="I99" s="45">
         <f>SUMPRODUCT((LEN(Consultas!$D$2:$D$1000)&gt;0)*(LEN(Consultas!$B$2:$B$1000)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A81" s="57" t="s">
-        <v>179</v>
-      </c>
-      <c r="B81" s="52"/>
-      <c r="C81" s="52"/>
-      <c r="D81" s="52"/>
-      <c r="E81" s="52"/>
-      <c r="F81" s="52"/>
-      <c r="G81" s="52"/>
-      <c r="H81" s="52"/>
-      <c r="I81" s="50">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" s="56" t="s">
+        <v>205</v>
+      </c>
+      <c r="B100" s="53"/>
+      <c r="C100" s="53"/>
+      <c r="D100" s="53"/>
+      <c r="E100" s="53"/>
+      <c r="F100" s="53"/>
+      <c r="G100" s="53"/>
+      <c r="H100" s="53"/>
+      <c r="I100" s="45">
         <f>SUMPRODUCT((Consultas!$H$2:$H$1000="Sí")*(Consultas!$F$2:$F$1000&lt;&gt;"GAM")*(Consultas!$F$2:$F$1000&lt;&gt;"Fuera de GAM"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A82" s="57" t="s">
-        <v>180</v>
-      </c>
-      <c r="B82" s="52"/>
-      <c r="C82" s="52"/>
-      <c r="D82" s="52"/>
-      <c r="E82" s="52"/>
-      <c r="F82" s="52"/>
-      <c r="G82" s="52"/>
-      <c r="H82" s="52"/>
-      <c r="I82" s="50">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" s="56" t="s">
+        <v>206</v>
+      </c>
+      <c r="B101" s="53"/>
+      <c r="C101" s="53"/>
+      <c r="D101" s="53"/>
+      <c r="E101" s="53"/>
+      <c r="F101" s="53"/>
+      <c r="G101" s="53"/>
+      <c r="H101" s="53"/>
+      <c r="I101" s="45">
         <f>SUMPRODUCT((Consultas!$J$2:$J$1000="Sí")*(Consultas!$H$2:$H$1000&lt;&gt;"Sí"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A83" s="57" t="s">
-        <v>181</v>
-      </c>
-      <c r="B83" s="52"/>
-      <c r="C83" s="52"/>
-      <c r="D83" s="52"/>
-      <c r="E83" s="52"/>
-      <c r="F83" s="52"/>
-      <c r="G83" s="52"/>
-      <c r="H83" s="52"/>
-      <c r="I83" s="50">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" s="56" t="s">
+        <v>207</v>
+      </c>
+      <c r="B102" s="53"/>
+      <c r="C102" s="53"/>
+      <c r="D102" s="53"/>
+      <c r="E102" s="53"/>
+      <c r="F102" s="53"/>
+      <c r="G102" s="53"/>
+      <c r="H102" s="53"/>
+      <c r="I102" s="45">
         <f>SUMPRODUCT((Consultas!$K$2:$K$1000="Sí")*(Consultas!$J$2:$J$1000&lt;&gt;"Sí"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A84" s="57" t="s">
-        <v>182</v>
-      </c>
-      <c r="B84" s="52"/>
-      <c r="C84" s="52"/>
-      <c r="D84" s="52"/>
-      <c r="E84" s="52"/>
-      <c r="F84" s="52"/>
-      <c r="G84" s="52"/>
-      <c r="H84" s="52"/>
-      <c r="I84" s="50">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" s="56" t="s">
+        <v>208</v>
+      </c>
+      <c r="B103" s="53"/>
+      <c r="C103" s="53"/>
+      <c r="D103" s="53"/>
+      <c r="E103" s="53"/>
+      <c r="F103" s="53"/>
+      <c r="G103" s="53"/>
+      <c r="H103" s="53"/>
+      <c r="I103" s="45">
         <f>SUMPRODUCT((Consultas!$K$2:$K$1000="Sí")*(LEN(Consultas!$L$2:$L$1000)=0))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A85" s="57" t="s">
-        <v>183</v>
-      </c>
-      <c r="B85" s="52"/>
-      <c r="C85" s="52"/>
-      <c r="D85" s="52"/>
-      <c r="E85" s="52"/>
-      <c r="F85" s="52"/>
-      <c r="G85" s="52"/>
-      <c r="H85" s="52"/>
-      <c r="I85" s="50">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" s="56" t="s">
+        <v>209</v>
+      </c>
+      <c r="B104" s="53"/>
+      <c r="C104" s="53"/>
+      <c r="D104" s="53"/>
+      <c r="E104" s="53"/>
+      <c r="F104" s="53"/>
+      <c r="G104" s="53"/>
+      <c r="H104" s="53"/>
+      <c r="I104" s="45">
         <f>SUMPRODUCT((LEN(Consultas!$L$2:$L$1000)&gt;0)*(Consultas!$K$2:$K$1000&lt;&gt;"Sí"))</f>
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A86" s="57" t="s">
-        <v>184</v>
-      </c>
-      <c r="B86" s="52"/>
-      <c r="C86" s="52"/>
-      <c r="D86" s="52"/>
-      <c r="E86" s="52"/>
-      <c r="F86" s="52"/>
-      <c r="G86" s="52"/>
-      <c r="H86" s="52"/>
-      <c r="I86" s="20">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" s="56" t="s">
+        <v>210</v>
+      </c>
+      <c r="B105" s="53"/>
+      <c r="C105" s="53"/>
+      <c r="D105" s="53"/>
+      <c r="E105" s="53"/>
+      <c r="F105" s="53"/>
+      <c r="G105" s="53"/>
+      <c r="H105" s="53"/>
+      <c r="I105" s="45">
+        <f>SUMPRODUCT((LEN(Consultas!$D$2:$D$1000)&gt;0)*(LEN(Consultas!$C$2:$C$1000)=0))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" s="56" t="s">
+        <v>211</v>
+      </c>
+      <c r="B106" s="53"/>
+      <c r="C106" s="53"/>
+      <c r="D106" s="53"/>
+      <c r="E106" s="53"/>
+      <c r="F106" s="53"/>
+      <c r="G106" s="53"/>
+      <c r="H106" s="53"/>
+      <c r="I106" s="20">
         <f>COUNTIF(Consultas!$G$2:$G$1000,"Sí")</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A33:H33"/>
+  <mergeCells count="18">
     <mergeCell ref="B6:K6"/>
-    <mergeCell ref="A80:H80"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A79:H79"/>
-    <mergeCell ref="B36:K36"/>
-    <mergeCell ref="A34:H34"/>
-    <mergeCell ref="B45:K45"/>
-    <mergeCell ref="A84:H84"/>
-    <mergeCell ref="A83:H83"/>
-    <mergeCell ref="A35:H35"/>
-    <mergeCell ref="A86:H86"/>
-    <mergeCell ref="A81:H81"/>
-    <mergeCell ref="A82:H82"/>
-    <mergeCell ref="A85:H85"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A102:H102"/>
+    <mergeCell ref="B64:K64"/>
+    <mergeCell ref="A100:H100"/>
+    <mergeCell ref="A101:H101"/>
+    <mergeCell ref="A106:H106"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A48:K48"/>
+    <mergeCell ref="A105:H105"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A51:H51"/>
+    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A99:H99"/>
+    <mergeCell ref="A103:H103"/>
+    <mergeCell ref="A98:H98"/>
+    <mergeCell ref="A104:H104"/>
+    <mergeCell ref="B55:K55"/>
   </mergeCells>
   <conditionalFormatting sqref="B6">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>SUM($I$79:$I$85)&gt;0</formula>
+    <cfRule type="expression" dxfId="2" priority="3">
+      <formula>SUM($I$98:$I$105)&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I79:I85">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>I79&gt;0</formula>
+  <conditionalFormatting sqref="I47">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>I47&lt;&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="6">
+  <conditionalFormatting sqref="I98:I105">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>I98&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="7">
     <dataValidation type="date" allowBlank="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Escribí la fecha como dd/mm/aaaa." sqref="B4:B5 F26:F29" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>DATE(2026,1,1)</formula1>
       <formula2>DATE(2030,12,31)</formula2>
@@ -9966,14 +10734,17 @@
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Alcance no válido" error="Número entero de cuentas o personas alcanzadas." promptTitle="Alcance (Insights)" prompt="Total de cuentas o personas alcanzadas en esa plataforma, no reproducciones. Vacía si la pieza no se publicó ahí o no hay dato." sqref="B26:D29" xr:uid="{00000000-0002-0000-0300-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí Sí o No." promptTitle="Condición" prompt="Elegí Sí o No." sqref="I32 I33 I34 I35" xr:uid="{00000000-0002-0000-0300-000004000000}">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Monto no válido" error="Solo números en colones." promptTitle="Pauta sin código" prompt="Solo anuncios que NO usan una pieza con código (por ejemplo, anuncios con foto), en las fechas Desde/Hasta. Vacía = sin pauta." sqref="H42" xr:uid="{00000000-0002-0000-0300-000004000000}">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Valor no válido" error="Elegí Sí o No." promptTitle="Condición" prompt="Elegí Sí o No." sqref="I51 I52 I53 I54" xr:uid="{00000000-0002-0000-0300-000005000000}">
       <formula1>"Sí,No"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Escribí la fecha como dd/mm/aaaa." promptTitle="Fecha de publicación" prompt="Día en que se publicó la pieza (dd/mm/aaaa)." sqref="B42:B43" xr:uid="{00000000-0002-0000-0300-000005000000}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Fecha no válida" error="Escribí la fecha como dd/mm/aaaa." promptTitle="Fecha de publicación" prompt="Día en que se publicó la pieza (dd/mm/aaaa)." sqref="B61:B62" xr:uid="{00000000-0002-0000-0300-000006000000}">
       <formula1>DATE(2026,1,1)</formula1>
       <formula2>DATE(2030,12,31)</formula2>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Alcance no válido" error="Número entero de cuentas o personas alcanzadas." promptTitle="Alcance en la ventana" prompt="Cuentas o personas alcanzadas por la pieza, sumando sus plataformas, leído el día «Cuenta hasta». Vacía si no hay dato." sqref="J42:J43" xr:uid="{00000000-0002-0000-0300-000006000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Alcance no válido" error="Número entero de cuentas o personas alcanzadas." promptTitle="Alcance en la ventana" prompt="Cuentas o personas alcanzadas por la pieza, sumando sus plataformas, leído el día «Cuenta hasta». Vacía si no hay dato." sqref="J61:J62" xr:uid="{00000000-0002-0000-0300-000007000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>